<commit_message>
updated code and results. T=20 and new board
</commit_message>
<xml_diff>
--- a/filter-cases/final_img/3x3/metrics_3x3.xlsx
+++ b/filter-cases/final_img/3x3/metrics_3x3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\fysiko_apth\ptuxiaki\thesis-cases\final_img\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\fysiko_apth\ptuxiaki\thesis-cases\final_img\3x3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F17019D-D9DC-4312-A07C-AE2D975BF53C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F89A2CE-86A4-46EE-854D-24B4EBC21A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30132" yWindow="588" windowWidth="23040" windowHeight="11976" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
+    <workbookView xWindow="-30108" yWindow="2892" windowWidth="16728" windowHeight="9828" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -768,10 +768,10 @@
         <v>28</v>
       </c>
       <c r="I8">
-        <v>535</v>
+        <v>2342</v>
       </c>
       <c r="J8">
-        <v>1044</v>
+        <v>6092</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -780,7 +780,7 @@
         <v>0</v>
       </c>
       <c r="M8">
-        <v>6</v>
+        <v>6.59</v>
       </c>
       <c r="N8">
         <v>737</v>
@@ -794,18 +794,18 @@
       </c>
       <c r="Q8">
         <f>1000/(T8-M8)</f>
-        <v>142.85714285714286</v>
+        <v>74.57121551081282</v>
       </c>
       <c r="R8">
         <f>U8*Q8</f>
-        <v>142.85714285714286</v>
+        <v>74.57121551081282</v>
       </c>
       <c r="S8">
         <f>Q8*10^6/P8</f>
-        <v>809.16427086612134</v>
+        <v>422.3825425848508</v>
       </c>
       <c r="T8">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="U8">
         <v>1</v>
@@ -837,19 +837,19 @@
         <v>28</v>
       </c>
       <c r="I9">
-        <v>10154</v>
+        <v>10027</v>
       </c>
       <c r="J9">
-        <v>6770</v>
+        <v>6716</v>
       </c>
       <c r="K9">
         <v>0</v>
       </c>
       <c r="L9">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="M9">
-        <v>0.68200000000000005</v>
+        <v>0.49299999999999999</v>
       </c>
       <c r="N9">
         <v>741</v>
@@ -863,18 +863,18 @@
       </c>
       <c r="Q9">
         <f>1000/(T9-M9)</f>
-        <v>81.182010066569248</v>
+        <v>51.263648946532008</v>
       </c>
       <c r="R9">
         <f>U9*Q9</f>
-        <v>81.182010066569248</v>
+        <v>51.263648946532008</v>
       </c>
       <c r="S9">
         <f>Q9*10^6/P9</f>
-        <v>459.8166559988743</v>
+        <v>290.3584133179952</v>
       </c>
       <c r="T9">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="U9">
         <v>1</v>
@@ -906,7 +906,7 @@
         <v>51.447336220525997</v>
       </c>
       <c r="I11">
-        <v>2320</v>
+        <v>2317</v>
       </c>
       <c r="J11">
         <v>6093</v>
@@ -918,7 +918,7 @@
         <v>0</v>
       </c>
       <c r="M11">
-        <v>4.6230000000000002</v>
+        <v>6.58</v>
       </c>
       <c r="N11">
         <v>737</v>
@@ -932,18 +932,18 @@
       </c>
       <c r="Q11">
         <f>1000/(T11-M11)</f>
-        <v>119.37447773665991</v>
+        <v>74.515648286140092</v>
       </c>
       <c r="R11">
         <f t="shared" ref="R11" si="0">U11*Q11</f>
-        <v>119.37447773665991</v>
+        <v>74.515648286140092</v>
       </c>
       <c r="S11">
         <f>Q11*10^6/P11</f>
-        <v>676.15493566465921</v>
+        <v>422.06780149499627</v>
       </c>
       <c r="T11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="U11">
         <v>1</v>
@@ -975,19 +975,19 @@
         <v>51.447336220525997</v>
       </c>
       <c r="I12">
-        <v>7739</v>
+        <v>21284</v>
       </c>
       <c r="J12">
-        <v>6565</v>
+        <v>13643</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="M12">
-        <v>1.101</v>
+        <v>4.7910000000000004</v>
       </c>
       <c r="N12">
         <v>742</v>
@@ -1001,18 +1001,18 @@
       </c>
       <c r="Q12">
         <f>1000/(T12-M12)</f>
-        <v>84.040675687032518</v>
+        <v>65.750542441975142</v>
       </c>
       <c r="R12">
         <f>U12*Q12</f>
-        <v>84.040675687032518</v>
+        <v>65.750542441975142</v>
       </c>
       <c r="S12">
         <f>Q12*10^6/P12</f>
-        <v>476.00550362513746</v>
+        <v>372.41038119767967</v>
       </c>
       <c r="T12">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="U12">
         <v>1</v>
@@ -1044,7 +1044,7 @@
         <v>40.931041264318701</v>
       </c>
       <c r="I14">
-        <v>4722</v>
+        <v>4720</v>
       </c>
       <c r="J14">
         <v>12233</v>
@@ -1056,7 +1056,7 @@
         <v>0</v>
       </c>
       <c r="M14">
-        <v>3.5950000000000002</v>
+        <v>5.7309999999999999</v>
       </c>
       <c r="N14">
         <v>1481</v>
@@ -1070,18 +1070,18 @@
       </c>
       <c r="Q14">
         <f t="shared" ref="Q14:Q15" si="2">1000/(T14-M14)</f>
-        <v>106.32642211589581</v>
+        <v>70.081995935244237</v>
       </c>
       <c r="R14">
         <f t="shared" ref="R14:R15" si="3">U14*Q14</f>
-        <v>106.32642211589581</v>
+        <v>70.081995935244237</v>
       </c>
       <c r="S14">
         <f t="shared" ref="S14:S15" si="4">Q14*10^6/P14</f>
-        <v>599.72148993979351</v>
+        <v>395.28913118534985</v>
       </c>
       <c r="T14">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="U14">
         <v>1</v>
@@ -1113,19 +1113,19 @@
         <v>40.931041264318701</v>
       </c>
       <c r="I15">
-        <v>17962</v>
+        <v>17837</v>
       </c>
       <c r="J15">
-        <v>13384</v>
+        <v>13331</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="M15">
-        <v>0.77200000000000002</v>
+        <v>0.48</v>
       </c>
       <c r="N15">
         <v>1490</v>
@@ -1139,18 +1139,18 @@
       </c>
       <c r="Q15">
         <f t="shared" si="2"/>
-        <v>81.779522407589141</v>
+        <v>51.229508196721312</v>
       </c>
       <c r="R15">
         <f t="shared" si="3"/>
-        <v>81.779522407589141</v>
+        <v>51.229508196721312</v>
       </c>
       <c r="S15">
         <f t="shared" si="4"/>
-        <v>461.24421838213408</v>
+        <v>288.93925729389019</v>
       </c>
       <c r="T15">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="U15">
         <v>1</v>

</xml_diff>